<commit_message>
Update paper-trade reports from Helius dry-run session.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,19 +37,23 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="009C5700"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="16"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,12 +67,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,9 +113,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -604,7 +613,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -614,7 +623,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -624,7 +633,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -634,7 +643,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -655,7 +664,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -666,7 +675,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>4.4</v>
+        <v>0.6000000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -676,7 +685,7 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>3.684889641</v>
+        <v>0.454962062</v>
       </c>
     </row>
     <row r="19">
@@ -686,7 +695,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>-0.7151103590000005</v>
+        <v>-0.1450379380000001</v>
       </c>
     </row>
     <row r="20">
@@ -715,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -800,51 +809,51 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Harry Potter flying car</t>
+          <t>wrappedape</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>wApe</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>-14.1%</t>
         </is>
       </c>
       <c r="F2" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="G2" s="12" t="n">
-        <v>0.193720911</v>
+        <v>0.166269841</v>
       </c>
       <c r="H2" s="12" t="n">
-        <v>-0.006279089000000015</v>
+        <v>-0.03373015900000001</v>
       </c>
       <c r="I2" s="10" t="inlineStr">
         <is>
-          <t>watchdog dead-coin 0.1% after 30s</t>
+          <t>trade-event stop-loss -14.1%</t>
         </is>
       </c>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>2VyRRmA2popb39MpxnXoBa4v7tj4YteJ5Yeu42rppump</t>
+          <t>CqZVFMMVxnz9VGENSXQLsRkJERsXWgR9iEy4gySypump</t>
         </is>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:33:45</t>
+          <t>2026-10-15 08:53:11</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:34:15</t>
+          <t>2026-10-15 08:53:11</t>
         </is>
       </c>
     </row>
@@ -854,51 +863,51 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Chinese RAM</t>
+          <t>PUMP</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>内存</t>
+          <t>PUMP</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>+5.9%</t>
+          <t>-16.3%</t>
         </is>
       </c>
       <c r="F3" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>0.204906978</v>
+        <v>0.161794524</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>0.004906977999999979</v>
+        <v>-0.03820547600000002</v>
       </c>
       <c r="I3" s="10" t="inlineStr">
         <is>
-          <t>watchdog dead-coin 5.9% after 30s</t>
+          <t>trade-event breakeven -16.3%</t>
         </is>
       </c>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>2U1gW43ea8QXqEQQcAPgZpdjPSjbTbS3Jh13k9hVpump</t>
+          <t>D58L4u1URrf1tMi6dRpG6rsnx1aDRDGNYqJiUPjhpump</t>
         </is>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:33:46</t>
+          <t>2026-10-15 08:53:12</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:34:16</t>
+          <t>2026-10-15 08:53:13</t>
         </is>
       </c>
     </row>
@@ -908,51 +917,51 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>toshiba</t>
+          <t>Marlboro</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>TOSHIBA</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+          <t>Headrush</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>LOST</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>-8.4%</t>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>-34.4%</t>
         </is>
       </c>
       <c r="F4" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>0.177354946</v>
+        <v>0.126897697</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>-0.022645054</v>
+        <v>-0.07310230300000001</v>
       </c>
       <c r="I4" s="10" t="inlineStr">
         <is>
-          <t>watchdog stop-loss -8.4%</t>
+          <t>watchdog stop-loss -34.4%</t>
         </is>
       </c>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>CxA5edLYZePQYJSZjPpL8LE9RrrBy6sV6JGpkkMHpump</t>
+          <t>A12KPqnVfVPH8pZCaBFDqYZdDNhqr5Qp3vcWkBiUpump</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:33:47</t>
+          <t>2026-10-15 08:53:15</t>
         </is>
       </c>
       <c r="L4" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:33:52</t>
+          <t>2026-10-15 08:53:17</t>
         </is>
       </c>
     </row>
@@ -962,53 +971,41 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Dolly</t>
+          <t>The Ozymandian Eagle</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Dolly</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>+2.9%</t>
-        </is>
-      </c>
+          <t>EAGLECOIN</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr"/>
       <c r="F5" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="12" t="n">
-        <v>0.967182157</v>
-      </c>
-      <c r="H5" s="12" t="n">
-        <v>-0.03281784300000001</v>
-      </c>
+      <c r="G5" s="10" t="inlineStr"/>
+      <c r="H5" s="10" t="inlineStr"/>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>trade-event trailing-stop 2.9% (-16.5% from peak)</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>FnyJBUbRq2q8sKLzgtgHj7tDquDEPK3HbR1KdVKzpump</t>
+          <t>55teXSXvAudgGEcPbAiw7CpExtMYbdtjFQNxwkSEpump</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:33:53</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:33:58</t>
-        </is>
-      </c>
+          <t>2026-10-15 08:53:21</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -1016,53 +1013,41 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Last One Standing</t>
+          <t>streamoors</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>LASTONE</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>+5.6%</t>
-        </is>
-      </c>
+          <t>STREAM</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr"/>
       <c r="F6" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G6" s="12" t="n">
-        <v>0.204304496</v>
-      </c>
-      <c r="H6" s="12" t="n">
-        <v>0.004304495999999991</v>
-      </c>
+      <c r="G6" s="10" t="inlineStr"/>
+      <c r="H6" s="10" t="inlineStr"/>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>watchdog dead-coin 5.6% after 30s</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>2bv7Hu2X7upuQwtSFjycegjaUJCx4dgxyixyFL9cX64f</t>
+          <t>FdsdBhh9RwZ4Wn3JBfjdppuU2PxMwaM7xYygdKxypump</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:34:17</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:47</t>
-        </is>
-      </c>
+          <t>2026-10-15 08:53:23</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
@@ -1070,272 +1055,44 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>LUMINOUS</t>
+          <t>good</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>LUMINOUS</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>-56.7%</t>
-        </is>
-      </c>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr"/>
       <c r="F7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>0.413221214</v>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>-0.586778786</v>
-      </c>
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="10" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr"/>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>trade-event breakeven -56.7%</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>Ki95qhKwtZrsZuq9YbVHwG3j9KMudhf5tKQ3QjEpump</t>
+          <t>4SRt4msD7kMa95YURo5p4YBSGFhNyL1WmYzJtQjBmGwy</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 07:34:19</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:50</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Webster</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>WEB</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>+0.1%</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>0.193594342</v>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>-0.006405658000000009</v>
-      </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>watchdog dead-coin 0.1% after 30s</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>68CBaJ9N5W8GtrxqxvgmoGgG9qALr5aV2RnT3tX7pump</t>
-        </is>
-      </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:20</t>
-        </is>
-      </c>
-      <c r="L8" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:50</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>NYC Horse Carriage Ban</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>WAN</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>+6.6%</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>0.206203184</v>
-      </c>
-      <c r="H9" s="12" t="n">
-        <v>0.006203184</v>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>watchdog dead-coin 6.6% after 30s</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>92WK6q3QA3PRBMZDYkix2DYv5WFV8QJ7ohcJtGqbpump</t>
-        </is>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:51</t>
-        </is>
-      </c>
-      <c r="L9" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:35:21</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Forced Runner</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Runner</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>-6.4%</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G10" s="12" t="n">
-        <v>0.181141959</v>
-      </c>
-      <c r="H10" s="12" t="n">
-        <v>-0.01885804100000002</v>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>trade-event breakeven -6.4%</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>FjUPh36x3raqf1CKJ9NTgQ3sHe5HmgBVFQnjMdeGpump</t>
-        </is>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:56</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>MAYA BLOOM</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>MAYA</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>+1.4%</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="12" t="n">
-        <v>0.943259454</v>
-      </c>
-      <c r="H11" s="12" t="n">
-        <v>-0.056740546</v>
-      </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>watchdog dead-coin 1.4% after 30s</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>HEhjFpMB389SMmPw3qaSW1rF9dStUQuczDvoaLp7pump</t>
-        </is>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:34:57</t>
-        </is>
-      </c>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 07:35:27</t>
-        </is>
-      </c>
+          <t>2026-10-15 08:53:24</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix SOL/USD price feed TLS and make holder lookups resilient.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$L$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,20 +37,20 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="009C5700"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C5700"/>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="16"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00006100"/>
     </font>
   </fonts>
   <fills count="6">
@@ -67,12 +67,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,15 +107,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -132,6 +132,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -613,7 +616,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -623,7 +626,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -633,7 +636,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -643,7 +646,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -653,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -664,7 +667,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -675,7 +678,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="18">
@@ -685,7 +688,7 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>0.454962062</v>
+        <v>0.449699276</v>
       </c>
     </row>
     <row r="19">
@@ -695,7 +698,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>-0.1450379380000001</v>
+        <v>0.04969927600000001</v>
       </c>
     </row>
     <row r="20">
@@ -724,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -809,53 +812,41 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>wrappedape</t>
+          <t>REAL CA IS ON TWEET READDD</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>wApe</t>
+          <t>READ</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>-14.1%</t>
-        </is>
-      </c>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr"/>
       <c r="F2" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G2" s="12" t="n">
-        <v>0.166269841</v>
-      </c>
-      <c r="H2" s="12" t="n">
-        <v>-0.03373015900000001</v>
-      </c>
+      <c r="G2" s="10" t="inlineStr"/>
+      <c r="H2" s="10" t="inlineStr"/>
       <c r="I2" s="10" t="inlineStr">
         <is>
-          <t>trade-event stop-loss -14.1%</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>CqZVFMMVxnz9VGENSXQLsRkJERsXWgR9iEy4gySypump</t>
+          <t>9jzimoanzEHKupPtj4EAVXmucwSjCQVr98TCGLAupump</t>
         </is>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:53:11</t>
-        </is>
-      </c>
-      <c r="L2" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 08:53:11</t>
-        </is>
-      </c>
+          <t>2026-10-15 08:58:53</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -863,51 +854,51 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>PUMP</t>
+          <t>Nihilism</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>PUMP</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="inlineStr">
+          <t>Nihilism</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>LOST</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>-16.3%</t>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>-6.3%</t>
         </is>
       </c>
       <c r="F3" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>0.161794524</v>
+        <v>0.181909038</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>-0.03820547600000002</v>
+        <v>-0.01809096200000002</v>
       </c>
       <c r="I3" s="10" t="inlineStr">
         <is>
-          <t>trade-event breakeven -16.3%</t>
+          <t>watchdog stop-loss -6.3%</t>
         </is>
       </c>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>D58L4u1URrf1tMi6dRpG6rsnx1aDRDGNYqJiUPjhpump</t>
+          <t>sW4r5TkA1vSMR6bjge82rXR1KNNsSJnvRWTikkbc8mS</t>
         </is>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:53:12</t>
+          <t>2026-10-15 08:58:54</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:53:13</t>
+          <t>2026-10-15 08:58:56</t>
         </is>
       </c>
     </row>
@@ -917,53 +908,41 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Marlboro</t>
+          <t>Dog Park</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Headrush</t>
+          <t>DOGPARK</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>-34.4%</t>
-        </is>
-      </c>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr"/>
       <c r="F4" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G4" s="12" t="n">
-        <v>0.126897697</v>
-      </c>
-      <c r="H4" s="12" t="n">
-        <v>-0.07310230300000001</v>
-      </c>
+      <c r="G4" s="10" t="inlineStr"/>
+      <c r="H4" s="10" t="inlineStr"/>
       <c r="I4" s="10" t="inlineStr">
         <is>
-          <t>watchdog stop-loss -34.4%</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>A12KPqnVfVPH8pZCaBFDqYZdDNhqr5Qp3vcWkBiUpump</t>
+          <t>BSFUrhXSc7tEkQ9aSaKFwTM8zBrwZEVdZV3jQGEETELE</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:53:15</t>
-        </is>
-      </c>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 08:53:17</t>
-        </is>
-      </c>
+          <t>2026-10-15 08:58:56</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -971,128 +950,56 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>The Ozymandian Eagle</t>
+          <t>CATECOIN</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>EAGLECOIN</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr"/>
+          <t>$CAT</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>+39.1%</t>
+        </is>
+      </c>
       <c r="F5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="10" t="inlineStr"/>
-      <c r="H5" s="10" t="inlineStr"/>
+        <v>0.2</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>0.267790238</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>0.067790238</v>
+      </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>holding</t>
+          <t>watchdog trailing-stop 39.1% (-48.3% from peak)</t>
         </is>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>55teXSXvAudgGEcPbAiw7CpExtMYbdtjFQNxwkSEpump</t>
+          <t>dxpPKBxotMDK3vXDAczw9SUSYkPdqrAujB9SAMkpump</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:53:21</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>streamoors</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>STREAM</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr"/>
-      <c r="F6" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G6" s="10" t="inlineStr"/>
-      <c r="H6" s="10" t="inlineStr"/>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>FdsdBhh9RwZ4Wn3JBfjdppuU2PxMwaM7xYygdKxypump</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 08:53:23</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr"/>
-      <c r="F7" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G7" s="10" t="inlineStr"/>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>4SRt4msD7kMa95YURo5p4YBSGFhNyL1WmYzJtQjBmGwy</t>
-        </is>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 08:53:24</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="inlineStr"/>
+          <t>2026-10-15 08:58:57</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 08:58:58</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:L5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1117,42 +1024,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Coin</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>LP tokens locked %</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Total liquidity USD</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Reasons</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>Top holder tokens</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Mint</t>
         </is>

</xml_diff>

<commit_message>
Retune dry-run pacing for the Helius Developer rate limits.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$L$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -115,7 +115,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -667,7 +667,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>0.449699276</v>
+        <v>0.650663157</v>
       </c>
     </row>
     <row r="19">
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>0.04969927600000001</v>
+        <v>-0.349336843</v>
       </c>
     </row>
     <row r="20">
@@ -727,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -812,12 +812,12 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>REAL CA IS ON TWEET READDD</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>READ</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -838,12 +838,12 @@
       </c>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>9jzimoanzEHKupPtj4EAVXmucwSjCQVr98TCGLAupump</t>
+          <t>4K2bzeQQmBPfJeSPh4MUBhf7MCX1iK35dh2Mjwrtpump</t>
         </is>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:58:53</t>
+          <t>2026-10-15 09:12:26</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr"/>
@@ -854,12 +854,12 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Nihilism</t>
+          <t>BYD</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>Nihilism</t>
+          <t>$BYD</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
@@ -869,36 +869,36 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>-6.3%</t>
+          <t>-51.4%</t>
         </is>
       </c>
       <c r="F3" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>0.181909038</v>
+        <v>0.093941554</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>-0.01809096200000002</v>
+        <v>-0.106058446</v>
       </c>
       <c r="I3" s="10" t="inlineStr">
         <is>
-          <t>watchdog stop-loss -6.3%</t>
+          <t>trade-event stop-loss -51.4%</t>
         </is>
       </c>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>sW4r5TkA1vSMR6bjge82rXR1KNNsSJnvRWTikkbc8mS</t>
+          <t>3zcRy61grA6KCrxKLnHz3kFsj6DghRxCwa1Zhjmrpump</t>
         </is>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:58:54</t>
+          <t>2026-10-15 09:12:29</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:58:56</t>
+          <t>2026-10-15 09:12:29</t>
         </is>
       </c>
     </row>
@@ -908,12 +908,12 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Dog Park</t>
+          <t>Discord Mod</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>DOGPARK</t>
+          <t>DiscMod</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>BSFUrhXSc7tEkQ9aSaKFwTM8zBrwZEVdZV3jQGEETELE</t>
+          <t>9dnTGSKS1q1hv2stduthT5Ph2JVC9Jsh8Fj2bgeTpump</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:58:56</t>
+          <t>2026-10-15 09:12:30</t>
         </is>
       </c>
       <c r="L4" s="10" t="inlineStr"/>
@@ -950,56 +950,218 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>CATECOIN</t>
+          <t>test</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>$CAT</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>+39.1%</t>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>-4.9%</t>
         </is>
       </c>
       <c r="F5" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>0.267790238</v>
+        <v>0.183843211</v>
       </c>
       <c r="H5" s="12" t="n">
-        <v>0.067790238</v>
+        <v>-0.016156789</v>
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>watchdog trailing-stop 39.1% (-48.3% from peak)</t>
+          <t>trade-event breakeven -4.9%</t>
         </is>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>dxpPKBxotMDK3vXDAczw9SUSYkPdqrAujB9SAMkpump</t>
+          <t>8AmrN25dYemThizkG6qjcdthvgYrnZcHvBPVZKqSpump</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:58:57</t>
+          <t>2026-10-15 09:12:32</t>
         </is>
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:58:58</t>
+          <t>2026-10-15 09:12:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>BOTCOIN</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>$BOT</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>-69.6%</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>0.058812368</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>-0.141187632</v>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>trade-event stop-loss -69.6%</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>4DuqSQqow3uHEDukrXh53FTckMWHifPR6NCShNigpump</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:12:41</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:12:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>+6.2%</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>0.111060535</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>-0.08893946500000001</v>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>watchdog trailing-stop 6.2% (-48.3% from peak)</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>3siM9nfVBRCvN2WS2rthbvX9Dm68jMchkxthvT4Wpump</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:12:45</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:12:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Doomed Rocket</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>DOOROC</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>+4.9%</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>0.203005489</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>0.003005489</v>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>watchdog trailing-stop 4.9% (-24.4% from peak)</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>HwiEQtx6xfNZvp73j6AmDQ8mYGvSaS2q2jeR3Huipump</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:12:47</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:12:48</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Track per-trade MFE/MAE excursions in the paper-trade report.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +37,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C5700"/>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -45,7 +45,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00006100"/>
+      <color rgb="009C5700"/>
     </font>
     <font>
       <b val="1"/>
@@ -67,7 +67,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -77,7 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +113,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -667,47 +667,71 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Total invested (SOL)</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>1</v>
+          <t>Avg peak (MFE)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>+41.4%</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Total back (SOL)</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>0.650663157</v>
+          <t>Avg drawdown (MAE)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>-17.0%</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Net P&amp;L (SOL)</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>-0.349336843</v>
+          <t>Total invested (SOL)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Total back (SOL)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>1.053916809</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Net P&amp;L (SOL)</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>-0.1460831910000002</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>Excel file</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>D:\AI\solana-trading-bot\reports\pumpfun_trades.xlsx</t>
         </is>
@@ -727,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -735,13 +759,15 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -772,35 +798,45 @@
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
+          <t>MFE %</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>MAE %</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
           <t>Invested SOL</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Exit SOL</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Profit/Loss SOL</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Mint</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Bought at</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>Sold at</t>
         </is>
@@ -812,41 +848,63 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Biscuit</t>
+          <t>Nihl</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Biscuit</t>
+          <t>NIHL</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr"/>
-      <c r="F2" s="12" t="n">
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>+3.3%</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>+6.7%</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G2" s="10" t="inlineStr"/>
-      <c r="H2" s="10" t="inlineStr"/>
-      <c r="I2" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="J2" s="10" t="inlineStr">
-        <is>
-          <t>4K2bzeQQmBPfJeSPh4MUBhf7MCX1iK35dh2Mjwrtpump</t>
-        </is>
+      <c r="I2" s="12" t="n">
+        <v>0.199762023</v>
+      </c>
+      <c r="J2" s="12" t="n">
+        <v>-0.0002379770000000003</v>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:26</t>
-        </is>
-      </c>
-      <c r="L2" s="10" t="inlineStr"/>
+          <t>watchdog dead-coin 3.3% after 30s</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="inlineStr">
+        <is>
+          <t>2EgByTVv7GQqCGSiQhEtQ4io2h4UmPSkZYbr2pTUpump</t>
+        </is>
+      </c>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:22</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:52</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -854,12 +912,12 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>BYD</t>
+          <t>UNUS SED LEO</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>$BYD</t>
+          <t>LÉO</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
@@ -869,36 +927,46 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>-51.4%</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n">
+          <t>-50.7%</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>-50.7%</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G3" s="12" t="n">
-        <v>0.093941554</v>
-      </c>
-      <c r="H3" s="12" t="n">
-        <v>-0.106058446</v>
-      </c>
-      <c r="I3" s="10" t="inlineStr">
-        <is>
-          <t>trade-event stop-loss -51.4%</t>
-        </is>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>3zcRy61grA6KCrxKLnHz3kFsj6DghRxCwa1Zhjmrpump</t>
-        </is>
+      <c r="I3" s="12" t="n">
+        <v>0.09529591499999999</v>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>-0.104704085</v>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:29</t>
+          <t>trade-event stop-loss -50.7%</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:29</t>
+          <t>6DYL4Eb3u49rDYDBiP7Pt4nCUQ7k4E15wjBkhmd8pump</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:25</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:25</t>
         </is>
       </c>
     </row>
@@ -908,41 +976,43 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Discord Mod</t>
+          <t>PSI</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>DiscMod</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
+          <t>PSI</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr"/>
-      <c r="F4" s="12" t="n">
+      <c r="E4" s="14" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="9" t="inlineStr"/>
+      <c r="H4" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G4" s="10" t="inlineStr"/>
-      <c r="H4" s="10" t="inlineStr"/>
-      <c r="I4" s="10" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr"/>
+      <c r="J4" s="10" t="inlineStr"/>
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>holding</t>
         </is>
       </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>9dnTGSKS1q1hv2stduthT5Ph2JVC9Jsh8Fj2bgeTpump</t>
-        </is>
-      </c>
-      <c r="K4" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:12:30</t>
-        </is>
-      </c>
-      <c r="L4" s="10" t="inlineStr"/>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>DAfUDBqZLtghKRjnGryHT5ic7mGmBo2b7feyvrhipump</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:27</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -950,12 +1020,12 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>Chaotic Rocket</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>CHAROC</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -965,36 +1035,46 @@
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>-4.9%</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="n">
+          <t>-51.3%</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>+0.5%</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>-51.3%</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="12" t="n">
-        <v>0.183843211</v>
-      </c>
-      <c r="H5" s="12" t="n">
-        <v>-0.016156789</v>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>trade-event breakeven -4.9%</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>8AmrN25dYemThizkG6qjcdthvgYrnZcHvBPVZKqSpump</t>
-        </is>
+      <c r="I5" s="12" t="n">
+        <v>0.09412549200000001</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-0.105874508</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:32</t>
+          <t>watchdog stop-loss -51.3%</t>
         </is>
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:39</t>
+          <t>HrvV3ubuY2rWgdYPc1tfTgE6MzwVop6uTN4vLtV1pump</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:29</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:31</t>
         </is>
       </c>
     </row>
@@ -1004,51 +1084,61 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>BOTCOIN</t>
+          <t>TRUMPISM</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>$BOT</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>-69.6%</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="n">
+          <t>$TRMPSM</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>+0.6%</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>+132.0%</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G6" s="12" t="n">
-        <v>0.058812368</v>
-      </c>
-      <c r="H6" s="12" t="n">
-        <v>-0.141187632</v>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>trade-event stop-loss -69.6%</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>4DuqSQqow3uHEDukrXh53FTckMWHifPR6NCShNigpump</t>
-        </is>
+      <c r="I6" s="12" t="n">
+        <v>0.194717265</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>-0.005282735000000011</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:41</t>
+          <t>watchdog trailing-stop 0.6% (-56.6% from peak)</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:41</t>
+          <t>C4zPh1LoacouSFyusuJDVAukKKGmPJnGW9j35F9ypump</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:33</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:35</t>
         </is>
       </c>
     </row>
@@ -1058,51 +1148,61 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Super General Robot</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>WON</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>+6.2%</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="n">
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>+39.1%</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>+75.8%</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G7" s="12" t="n">
-        <v>0.111060535</v>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>-0.08893946500000001</v>
-      </c>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>watchdog trailing-stop 6.2% (-48.3% from peak)</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>3siM9nfVBRCvN2WS2rthbvX9Dm68jMchkxthvT4Wpump</t>
-        </is>
+      <c r="I7" s="12" t="n">
+        <v>0.268779474</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0.06877947400000001</v>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:45</t>
+          <t>watchdog trailing-stop 39.1% (-20.9% from peak)</t>
         </is>
       </c>
       <c r="L7" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:45</t>
+          <t>6zLWahuStCZCVjgFc1gwPZ6dE9vkjoswWysKrHQ9pump</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:40</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:41</t>
         </is>
       </c>
     </row>
@@ -1112,56 +1212,154 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Doomed Rocket</t>
+          <t>@k</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>DOOROC</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
+          <t>@K</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>WON</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>+4.9%</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="n">
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>+4.0%</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>+33.1%</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="G8" s="12" t="n">
-        <v>0.203005489</v>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>0.003005489</v>
-      </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>watchdog trailing-stop 4.9% (-24.4% from peak)</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>HwiEQtx6xfNZvp73j6AmDQ8mYGvSaS2q2jeR3Huipump</t>
-        </is>
+      <c r="I8" s="12" t="n">
+        <v>0.20123664</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>0.001236639999999983</v>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:47</t>
+          <t>watchdog trailing-stop 4.0% (-21.9% from peak)</t>
         </is>
       </c>
       <c r="L8" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:12:48</t>
-        </is>
-      </c>
+          <t>8NVp9cQZug3a8gLjqBsqrffwtgqjy6HJVdScxRPBpump</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:44</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Bonsai</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Bonsai</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I9" s="10" t="inlineStr"/>
+      <c r="J9" s="10" t="inlineStr"/>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>26uP3eBS2zCvNGduhou2uTPQvydtrdFKxaVBznpmpump</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:53</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>The Bitcoin Cat</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>TheCat</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="9" t="inlineStr"/>
+      <c r="H10" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="10" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>6xMShQxQpPcXxBUUX7hxvGiYJHsohgEYJz6woNvVpump</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:17:54</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:N10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Auto-save bot updates 2026-10-15 09:35
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,15 +45,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C5700"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -73,11 +69,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,9 +98,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,9 +123,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -616,7 +604,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -626,7 +614,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -636,7 +624,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -646,7 +634,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -656,7 +644,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -667,7 +655,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
@@ -679,7 +667,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+41.4%</t>
+          <t>+5.7%</t>
         </is>
       </c>
     </row>
@@ -691,7 +679,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>-17.0%</t>
+          <t>-4.1%</t>
         </is>
       </c>
     </row>
@@ -702,7 +690,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="20">
@@ -712,7 +700,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1.053916809</v>
+        <v>0.7419586140000001</v>
       </c>
     </row>
     <row r="21">
@@ -722,7 +710,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>-0.1460831910000002</v>
+        <v>-0.05804138599999997</v>
       </c>
     </row>
     <row r="22">
@@ -751,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -848,12 +836,12 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Nihl</t>
+          <t>HE HAS A CONFIRMED WALLET???</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>NIHL</t>
+          <t>Nihilism</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -863,12 +851,12 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>+3.3%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>+6.7%</t>
+          <t>+1.3%</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -880,29 +868,29 @@
         <v>0.2</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.199762023</v>
+        <v>0.193466246</v>
       </c>
       <c r="J2" s="12" t="n">
-        <v>-0.0002379770000000003</v>
+        <v>-0.006533754000000003</v>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>watchdog dead-coin 3.3% after 30s</t>
+          <t>watchdog dead-coin 0.0% after 30s</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>2EgByTVv7GQqCGSiQhEtQ4io2h4UmPSkZYbr2pTUpump</t>
+          <t>HYFhhCTgzKNwjDWgNXQGPiNXyRgTojhYhDPf3ZTbpump</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:17:22</t>
+          <t>2026-10-15 09:32:42</t>
         </is>
       </c>
       <c r="N2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:17:52</t>
+          <t>2026-10-15 09:33:12</t>
         </is>
       </c>
     </row>
@@ -912,22 +900,22 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>UNUS SED LEO</t>
+          <t>HE HAS A CONFIRMED WALLET???</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>LÉO</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>-50.7%</t>
+          <t>Nihilism</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
@@ -937,36 +925,36 @@
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>-50.7%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="H3" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09529591499999999</v>
+        <v>0.193466246</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>-0.104704085</v>
+        <v>-0.006533754000000003</v>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>trade-event stop-loss -50.7%</t>
+          <t>watchdog dead-coin 0.0% after 30s</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>6DYL4Eb3u49rDYDBiP7Pt4nCUQ7k4E15wjBkhmd8pump</t>
+          <t>7VYnAe6TBHijsr3rW2TxhVcTAjvVFFBXTnfZrXsEpump</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:17:25</t>
+          <t>2026-10-15 09:32:43</t>
         </is>
       </c>
       <c r="N3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:17:25</t>
+          <t>2026-10-15 09:33:13</t>
         </is>
       </c>
     </row>
@@ -976,43 +964,63 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>PSI</t>
+          <t>HE HAS A CONFIRMED WALLET???</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>PSI</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
-      <c r="G4" s="9" t="inlineStr"/>
+          <t>Nihilism</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
       <c r="H4" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="I4" s="10" t="inlineStr"/>
-      <c r="J4" s="10" t="inlineStr"/>
+      <c r="I4" s="12" t="n">
+        <v>0.193466246</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>-0.006533754000000003</v>
+      </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>holding</t>
+          <t>watchdog dead-coin 0.0% after 30s</t>
         </is>
       </c>
       <c r="L4" s="10" t="inlineStr">
         <is>
-          <t>DAfUDBqZLtghKRjnGryHT5ic7mGmBo2b7feyvrhipump</t>
+          <t>8tKTLE9JG2KkW1ry1tGbZNquRQFhK2RTAamKGiMVpump</t>
         </is>
       </c>
       <c r="M4" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:17:27</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="inlineStr"/>
+          <t>2026-10-15 09:32:45</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:33:15</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -1020,12 +1028,12 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Chaotic Rocket</t>
+          <t>fork it to ya</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>CHAROC</t>
+          <t>forkya</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -1035,331 +1043,51 @@
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>-51.3%</t>
+          <t>-16.5%</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>+0.5%</t>
+          <t>+21.6%</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>-51.3%</t>
+          <t>-16.5%</t>
         </is>
       </c>
       <c r="H5" s="12" t="n">
         <v>0.2</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>0.09412549200000001</v>
+        <v>0.161559876</v>
       </c>
       <c r="J5" s="12" t="n">
-        <v>-0.105874508</v>
+        <v>-0.03844012400000002</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>watchdog stop-loss -51.3%</t>
+          <t>watchdog breakeven -16.5%</t>
         </is>
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>HrvV3ubuY2rWgdYPc1tfTgE6MzwVop6uTN4vLtV1pump</t>
+          <t>4MTRYyKdXDP5FJKWARKMBYPKLPHzRbNC9vgLp7Lppump</t>
         </is>
       </c>
       <c r="M5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:17:29</t>
+          <t>2026-10-15 09:33:15</t>
         </is>
       </c>
       <c r="N5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:17:31</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>TRUMPISM</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>$TRMPSM</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>+0.6%</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>+132.0%</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>0.194717265</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>-0.005282735000000011</v>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>watchdog trailing-stop 0.6% (-56.6% from peak)</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>C4zPh1LoacouSFyusuJDVAukKKGmPJnGW9j35F9ypump</t>
-        </is>
-      </c>
-      <c r="M6" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:33</t>
-        </is>
-      </c>
-      <c r="N6" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:35</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Super General Robot</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>+39.1%</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>+75.8%</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <v>0.268779474</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>0.06877947400000001</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>watchdog trailing-stop 39.1% (-20.9% from peak)</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>6zLWahuStCZCVjgFc1gwPZ6dE9vkjoswWysKrHQ9pump</t>
-        </is>
-      </c>
-      <c r="M7" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:40</t>
-        </is>
-      </c>
-      <c r="N7" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:41</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>@k</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>@K</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>+4.0%</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>+33.1%</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I8" s="12" t="n">
-        <v>0.20123664</v>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>0.001236639999999983</v>
-      </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>watchdog trailing-stop 4.0% (-21.9% from peak)</t>
-        </is>
-      </c>
-      <c r="L8" s="10" t="inlineStr">
-        <is>
-          <t>8NVp9cQZug3a8gLjqBsqrffwtgqjy6HJVdScxRPBpump</t>
-        </is>
-      </c>
-      <c r="M8" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:44</t>
-        </is>
-      </c>
-      <c r="N8" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:50</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Bonsai</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Bonsai</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I9" s="10" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L9" s="10" t="inlineStr">
-        <is>
-          <t>26uP3eBS2zCvNGduhou2uTPQvydtrdFKxaVBznpmpump</t>
-        </is>
-      </c>
-      <c r="M9" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:53</t>
-        </is>
-      </c>
-      <c r="N9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>The Bitcoin Cat</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>TheCat</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
-      <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I10" s="10" t="inlineStr"/>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>6xMShQxQpPcXxBUUX7hxvGiYJHsohgEYJz6woNvVpump</t>
-        </is>
-      </c>
-      <c r="M10" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:17:54</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="inlineStr"/>
+          <t>2026-10-15 09:33:16</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N10"/>
+  <autoFilter ref="A1:N5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1384,42 +1112,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Coin</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>LP tokens locked %</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Total liquidity USD</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>Reasons</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Top holder tokens</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>Mint</t>
         </is>

</xml_diff>

<commit_message>
Gate entries on sell pressure, not just gross buy volume
The confirm window only ever accumulated buy volume, so MIN_CONFIRM_BUY_SOL could be
satisfied by the deployer plus a couple of bots -- and then sold into. Track the sell
side too and reject launches where more money is leaving than arriving, which is the
population that goes flat and then bleeds.

- confirm.py: Candidate records sell_sol and derives net_buy_sol / sell_ratio.
- config.py: MIN_CONFIRM_NET_SOL and MAX_CONFIRM_SELL_RATIO, both off (0) by default
  so current behaviour is unchanged until a sweep says otherwise.
- interleaved_sweep.py: 'pressure' schedule (off / net>=1 / ratio<=0.5 / both).
- test_graduation_fix.py: covers the dump case a gross-buy gate lets through.

Also adds the diagnostics used for this analysis under tools/_*.py.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -670,7 +670,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>86.7%</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+93.5%</t>
+          <t>+118.2%</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>15.791703366</v>
+        <v>22.10382535</v>
       </c>
     </row>
     <row r="21">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>3.791703366</v>
+        <v>7.103825350000001</v>
       </c>
     </row>
     <row r="22">
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1307,22 +1307,38 @@
           <t>Hugo</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>+243.0%</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>+456.7%</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
       <c r="H9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="10" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
+      <c r="I9" s="12" t="n">
+        <v>3.42975081</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>2.42975081</v>
+      </c>
       <c r="K9" s="10" t="inlineStr">
         <is>
-          <t>holding</t>
+          <t>trade-event trailing-stop 284.1% (-31.0% from peak, tol=28%)</t>
         </is>
       </c>
       <c r="L9" s="10" t="inlineStr">
@@ -1335,7 +1351,11 @@
           <t>2026-10-15 21:53:12</t>
         </is>
       </c>
-      <c r="N9" s="10" t="inlineStr"/>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 21:56:45</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
@@ -1965,8 +1985,180 @@
       </c>
       <c r="N21" s="10" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Jeet Slapper</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>JSLAP</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>+4.2%</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>+9.8%</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>1.041772817</v>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>0.04177281700000002</v>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>watchdog dead-coin 9.8% after 30s</t>
+        </is>
+      </c>
+      <c r="L22" s="10" t="inlineStr">
+        <is>
+          <t>AjD35QUtwy6NieqkkAKKNacfzQVvdh47BR6pHr6Xpump</t>
+        </is>
+      </c>
+      <c r="M22" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 21:56:55</t>
+        </is>
+      </c>
+      <c r="N22" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 21:57:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Launch on Moat</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>MOAT</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>+84.1%</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>+184.7%</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="12" t="n">
+        <v>1.840598357</v>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>0.840598357</v>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>trade-event trailing-stop 102.8% (-28.8% from peak, tol=28%)</t>
+        </is>
+      </c>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>7bmhZEWfmGzrJC3xuK4pfUWrgzo1ymQ9X6wxzFPypump</t>
+        </is>
+      </c>
+      <c r="M23" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 21:57:48</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 21:57:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Official NeymarJr. Token</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>NEYMAR</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr"/>
+      <c r="F24" s="9" t="inlineStr"/>
+      <c r="G24" s="9" t="inlineStr"/>
+      <c r="H24" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="10" t="inlineStr"/>
+      <c r="J24" s="10" t="inlineStr"/>
+      <c r="K24" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L24" s="10" t="inlineStr">
+        <is>
+          <t>EN37FBT9sApUgGMtLiGmYEESR1E6JjqowidyQTF2pump</t>
+        </is>
+      </c>
+      <c r="M24" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15 21:57:52</t>
+        </is>
+      </c>
+      <c r="N24" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N21"/>
+  <autoFilter ref="A1:N24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Run the validation at a sample size worth believing
Every arm so far used 8-minute blocks, which yields 10-40 trades. That is not enough
to judge fat-tailed memecoin returns, where one 1000% trade can move a small sample's
mean by hundreds of points -- and it is why some earlier arms looked impressive on
numbers that did not deserve trust.

Measured rate is ~2 trades per minute of arm-time for a filtered arm, so this uses
30-minute blocks x 3 reps: roughly 180 trades per arm and three independent blocks.

- interleaved_sweep.py: 'final' schedule -- A-stack-off (live today), B-stack-press
  (adds sell-pressure guards), C-stack-full (adds the regime gate). B isolates the
  pressure filter, C isolates the gate on top. MIN_CONFIRM_BUY_SOL=2 in every arm so
  the comparison is about the new guards, not the level.
- report(): now prints median, win rate and mfe10 alongside the mean, because the mean
  alone is exactly what a lucky trade can fake.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -37,16 +37,16 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="009C5700"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="16"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -67,17 +67,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,15 +107,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -131,10 +131,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -623,7 +626,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -633,7 +636,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -643,7 +646,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -664,7 +667,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -676,7 +679,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>+29.7%</t>
         </is>
       </c>
     </row>
@@ -698,8 +701,8 @@
           <t>Total invested (SOL)</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
-        <v>0</v>
+      <c r="B19" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -708,8 +711,8 @@
           <t>Total back (SOL)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
-        <v>0</v>
+      <c r="B20" s="4" t="n">
+        <v>1.006577783</v>
       </c>
     </row>
     <row r="21">
@@ -719,7 +722,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>0</v>
+        <v>0.006577783000000004</v>
       </c>
     </row>
     <row r="22">
@@ -845,43 +848,63 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>LOFI</t>
+          <t>bum</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>LOFI</t>
+          <t>bum</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
-      <c r="G2" s="9" t="inlineStr"/>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>+0.7%</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>+29.7%</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
       <c r="H2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="10" t="inlineStr"/>
-      <c r="J2" s="10" t="inlineStr"/>
+      <c r="I2" s="12" t="n">
+        <v>1.006577783</v>
+      </c>
+      <c r="J2" s="12" t="n">
+        <v>0.006577783000000004</v>
+      </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>holding</t>
+          <t>watchdog trailing-stop 9.6% (-15.5% from peak, tol=10%)</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>EaCzZRVGhdBL9VsAwui7Wc8pSUqMz97Ht4PsWoLQpump</t>
+          <t>23tZw1ZMsRG2ZVWzBNWqFS8BCkNXcVyJcbt5ckakpump</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 22:00:41</t>
-        </is>
-      </c>
-      <c r="N2" s="10" t="inlineStr"/>
+          <t>2026-10-16 00:53:13</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 00:53:16</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -889,20 +912,20 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Cash Cat</t>
+          <t>PuzunSync</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>BLACKIE</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="inlineStr">
+          <t>PUZUN</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr"/>
+      <c r="E3" s="13" t="inlineStr"/>
       <c r="F3" s="9" t="inlineStr"/>
       <c r="G3" s="9" t="inlineStr"/>
       <c r="H3" s="12" t="n">
@@ -917,12 +940,12 @@
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>63AJe8VZuQ9JbQc6L1JAwFZLQmxEovihVJmL4ucnpump</t>
+          <t>BExLBBVqk4mVVyU1GMk8Y9ZK5k8hCAefpoPgocKppump</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 22:00:49</t>
+          <t>2026-10-16 00:53:22</t>
         </is>
       </c>
       <c r="N3" s="10" t="inlineStr"/>
@@ -931,14 +954,22 @@
       <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="10" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>OBSIDIAN</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr"/>
+      <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="9" t="inlineStr"/>
       <c r="G4" s="9" t="inlineStr"/>
       <c r="H4" s="12" t="n">
@@ -953,12 +984,12 @@
       </c>
       <c r="L4" s="10" t="inlineStr">
         <is>
-          <t>43ePcpnkHoE4yXhaq5e9uQTdxGqNrzwam1AhDqk9pump</t>
+          <t>4waSCsC6ppAxjAgVcLCiSVRX5L1Qv1zqTvAKkstkpump</t>
         </is>
       </c>
       <c r="M4" s="10" t="inlineStr">
         <is>
-          <t>2026-10-15 22:00:51</t>
+          <t>2026-10-16 00:53:24</t>
         </is>
       </c>
       <c r="N4" s="10" t="inlineStr"/>
@@ -989,80 +1020,80 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Coin</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>LP tokens locked %</t>
         </is>
       </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Total liquidity USD</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>Reasons</t>
         </is>
       </c>
-      <c r="G1" s="13" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Top holder tokens</t>
         </is>
       </c>
-      <c r="H1" s="13" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>Mint</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>2026-10-15 22:00:47</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>First Responders Coin</t>
-        </is>
-      </c>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>FRC</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="n">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-16 00:53:15</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Microducks</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>MICRODUCKS</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="n">
         <v>135.291892573446</v>
       </c>
-      <c r="E2" s="16" t="n">
+      <c r="E2" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=13 &gt; 5</t>
-        </is>
-      </c>
-      <c r="G2" s="16" t="n">
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=12 &gt; 5</t>
+        </is>
+      </c>
+      <c r="G2" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>GiUgf9yEPfQXhgCnX9pVvJgiQYbfUcPosg8uxMCSpump</t>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>FCUbf4HHAdGwrJpzmDT7PJfWWzuYqAyEwkGZLP6ypump</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add STONK liquidity comparables screen
Screens Jupiter's verified token set (3,987 tokens) for Solana tokens whose
DEX liquidity sits within 0.5x-2x of STONK (StonkFun token), reporting
liquidity, market cap, holders, organic score and mint/freeze authority.

Writes reports/stonk_liquidity_comps.json. Data only.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,7 +37,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="009C5700"/>
     </font>
     <font>
       <b val="1"/>
@@ -48,8 +48,12 @@
       <b val="1"/>
       <color rgb="00006100"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,12 +67,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,8 +114,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -601,7 +610,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -611,7 +620,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -621,7 +630,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -641,7 +650,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -664,7 +673,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+108.9%</t>
+          <t>+0.0%</t>
         </is>
       </c>
     </row>
@@ -676,7 +685,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>-2.1%</t>
+          <t>+0.0%</t>
         </is>
       </c>
     </row>
@@ -686,8 +695,8 @@
           <t>Total invested (SOL)</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
-        <v>1</v>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -696,8 +705,8 @@
           <t>Total back (SOL)</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>0.979319382</v>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -707,7 +716,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>-0.02068061799999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -736,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -833,66 +842,90 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>SATINU</t>
+          <t>Meme Index 100</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>SATINU</t>
+          <t>MEME100</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>-2.1%</t>
-        </is>
-      </c>
-      <c r="F2" s="9" t="inlineStr">
-        <is>
-          <t>+108.9%</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr">
-        <is>
-          <t>-2.1%</t>
-        </is>
-      </c>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="9" t="inlineStr"/>
       <c r="H2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="12" t="n">
-        <v>0.979319382</v>
-      </c>
-      <c r="J2" s="12" t="n">
-        <v>-0.02068061799999998</v>
-      </c>
+      <c r="I2" s="10" t="inlineStr"/>
+      <c r="J2" s="10" t="inlineStr"/>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>watchdog breakeven -2.1%</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>Cw3TfKqnvnsMGdYVm4kMFiowb2K5XXmR2vXYTxudpump</t>
+          <t>YsALHbPSQkSu53AQsAKCxKFVknAPpJ8Vr58GoyNpump</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 03:18:45</t>
-        </is>
-      </c>
-      <c r="N2" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 03:18:46</t>
-        </is>
-      </c>
+          <t>2026-10-16 03:31:49</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Rankz</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>RANKZ</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="9" t="inlineStr"/>
+      <c r="H3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="10" t="inlineStr"/>
+      <c r="J3" s="10" t="inlineStr"/>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>7d8W2JerSognHYeBAtcg2RaJs97rccUkAbR8KTVhpump</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 03:31:51</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N2"/>
+  <autoFilter ref="A1:N3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Egyptian Arabic voiceover renderer for the STONK case study
Renders the case study as ar-EG-SalmaNeural speech via edge-tts.
Injects truststore so TLS verification works behind Norton's
certificate interception. Output is a local mp3, not committed.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -41,16 +41,16 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="009C5700"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="16"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C0006"/>
     </font>
   </fonts>
   <fills count="6">
@@ -72,12 +72,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,14 +107,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -134,7 +134,13 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -613,7 +619,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -623,7 +629,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -633,7 +639,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -643,7 +649,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -653,7 +659,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -664,7 +670,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -676,7 +682,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+26.7%</t>
+          <t>+25.4%</t>
         </is>
       </c>
     </row>
@@ -688,7 +694,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-1.4%</t>
         </is>
       </c>
     </row>
@@ -699,7 +705,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -709,7 +715,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1.002599381</v>
+        <v>6.460753118</v>
       </c>
     </row>
     <row r="21">
@@ -719,7 +725,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>0.002599381000000012</v>
+        <v>0.4607531180000004</v>
       </c>
     </row>
     <row r="22">
@@ -748,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -919,20 +925,36 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
-      <c r="G3" s="9" t="inlineStr"/>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>-0.9%</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>+7.4%</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>-0.9%</t>
+        </is>
+      </c>
       <c r="H3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="10" t="inlineStr"/>
-      <c r="J3" s="10" t="inlineStr"/>
+      <c r="I3" s="12" t="n">
+        <v>0.991037663</v>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>-0.008962337000000042</v>
+      </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>holding</t>
+          <t>watchdog breakeven -0.9%</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
@@ -945,7 +967,11 @@
           <t>2026-10-16 04:39:54</t>
         </is>
       </c>
-      <c r="N3" s="10" t="inlineStr"/>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:39:56</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n">
@@ -963,36 +989,512 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
-      <c r="G4" s="9" t="inlineStr"/>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>-7.0%</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>-7.0%</t>
+        </is>
+      </c>
       <c r="H4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="10" t="inlineStr"/>
-      <c r="J4" s="10" t="inlineStr"/>
+      <c r="I4" s="12" t="n">
+        <v>0.930309045</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>-0.069690955</v>
+      </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
+          <t>watchdog stop-loss -7.0%</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>6N22dmEVa9Ky8ezvhm5FvCtTpFgd9fLBuSW9wSmwpump</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:39:55</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:39:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Toly $1 Coin</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="9" t="inlineStr"/>
+      <c r="H5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="10" t="inlineStr"/>
+      <c r="J5" s="10" t="inlineStr"/>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
           <t>holding</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>6N22dmEVa9Ky8ezvhm5FvCtTpFgd9fLBuSW9wSmwpump</t>
-        </is>
-      </c>
-      <c r="M4" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:39:55</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="inlineStr"/>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>2dwa82kTNo8MXvj3K8wZqsx79h97pTXC2nCAfTkYpump</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:10</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Flying tesla skyster</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>FTS</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="9" t="inlineStr"/>
+      <c r="H6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="10" t="inlineStr"/>
+      <c r="J6" s="10" t="inlineStr"/>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>3njQBDXmF4Z97u5BJzAzBRuMTMA89N3942i65pdLpump</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:13</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Baton Man</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>BatonMan</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>+30.1%</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>+48.5%</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>1.300951674</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0.300951674</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>watchdog trailing-stop 30.1% (-12.4% from peak, tol=10%)</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>8f6htt8WT2qGau2T7MBXMW9NJXpcfFhTetdrcS2Rpump</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:17</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Ava Larps</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Ava</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="9" t="inlineStr"/>
+      <c r="H8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="10" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>95yf3XvjpTzJfWAcqqvXhH5s4DS55tY1tiJ1iR9qpump</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:24</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>ТamPad</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>ТamPad</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="10" t="inlineStr"/>
+      <c r="J9" s="10" t="inlineStr"/>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>DiGYfgNSzYsvN4zbjZa6NyjyNE95X2qkV32ML5thpump</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:51</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>ТamPad</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>ТamPad</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>-1.8%</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>-0.8%</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>0.981940087</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>-0.01805991299999998</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>watchdog dead-coin -0.8% after 30s</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>FppJ8swha44WggXN2UG9mTKG1b35ACBUYhvMsdKWpump</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:56</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:41:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>amor</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>amor</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>+25.4%</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>+69.8%</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>1.253915268</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>0.2539152680000001</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>watchdog trailing-stop 25.4% (-26.2% from peak, tol=18%)</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>HuDj7pNgAcVXb7cEtPXJEQTqVQGQGkuHBTh7Djsopump</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:41:19</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:41:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>TESCREAL</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>TESCREAL</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="9" t="inlineStr"/>
+      <c r="H12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="10" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>NZZY9SnqrMLHiHxoqnstLCsF7Lmr1rGF1Ba3HAEpump</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:41:25</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>DRAINLOVE</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>DRAINLOVE</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="9" t="inlineStr"/>
+      <c r="H13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="10" t="inlineStr"/>
+      <c r="J13" s="10" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>holding</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>9HmC4jXxkaFchQHQEy873oA3bCcpGziz1hW7aP14pump</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:41:34</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N4"/>
+  <autoFilter ref="A1:N13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1003,7 +1505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1017,44 +1519,188 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Coin</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>LP tokens locked %</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Total liquidity USD</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Reasons</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>Top holder tokens</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Mint</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:39:57</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>SUPER INU</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>SINU</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="n">
+        <v>3.319804998249779</v>
+      </c>
+      <c r="E2" s="18" t="n">
+        <v>7919.615246532211</v>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 3.32% | 2- Total Locked Liquidity $7.9K | BLOCK insider-whale 763,701,068 tokens (&gt;= 100,000,000); concentrated-holder 76.4% &gt;= 30%</t>
+        </is>
+      </c>
+      <c r="G2" s="18" t="n">
+        <v>763701067.612466</v>
+      </c>
+      <c r="H2" s="16" t="inlineStr">
+        <is>
+          <t>3szhHxoagYbDNEEj35cmBxKr3iadFLrrSVyjjuwapump</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:12</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Phase Punk</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>PHASEPUNK</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="n">
+        <v>135.291892573446</v>
+      </c>
+      <c r="E3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=15 &gt; 5</t>
+        </is>
+      </c>
+      <c r="G3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>9KGZuyJ8UXokgREBFxGguA1hVVdUmBYwtTSaQbPMpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:19</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Up Side Down Tesla</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>135.291892573446</v>
+      </c>
+      <c r="E4" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK clone-ticker USDT; serial-deployer launches=38 &gt; 5</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>7vG48c29W1oAtAeUUpphLgQ2bDUWTiXokhrYF2zsX34p</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:40:41</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>niggi</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>niggi</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>135.291892573446</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=6 &gt; 5</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>3o1kTH57F6kuuhjcpMSuggQHRjxmThEri3iGnPXfpump</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden the test supervisor and add a go-live connectivity check
The program died twice more with no error of any kind -- no traceback, no antivirus
event, logs simply stop. Timing matched a Norton block warning. The launchers needed to
be more forgiving regardless of the cause:

- single-instance lock (reports/logs/program.lock) so repeated launches can never start
  two copies that fight over the same ports and log files.
- 6 attempts per stage instead of 4.
- exits early when program_complete.flag exists.

tools/check_connectivity.py tests both connections the bot needs -- HTTP RPC (buys and
sells) and the WebSocket trade stream (confirm window and trailing stop) -- with
retries, and prints no secrets. Run it before going live: a firewall silently eating
the trade stream would leave the bot blind while looking healthy.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,11 +37,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -67,12 +67,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,9 +113,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -138,9 +138,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -682,7 +682,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+25.4%</t>
+          <t>+72.7%</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>-1.4%</t>
+          <t>-2.1%</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>6.460753118</v>
+        <v>2.202809591</v>
       </c>
     </row>
     <row r="21">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>0.4607531180000004</v>
+        <v>0.2028095909999998</v>
       </c>
     </row>
     <row r="22">
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -851,61 +851,61 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>VEILTROLL</t>
+          <t>Okay</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>VEILTROLL</t>
+          <t>OKAY</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>+0.3%</t>
+          <t>-4.1%</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>+26.7%</t>
+          <t>+76.9%</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-4.1%</t>
         </is>
       </c>
       <c r="H2" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>1.002599381</v>
+        <v>0.958761799</v>
       </c>
       <c r="J2" s="12" t="n">
-        <v>0.002599381000000012</v>
+        <v>-0.04123820099999997</v>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>watchdog trailing-stop 0.3% (-20.9% from peak, tol=10%)</t>
+          <t>trade-event breakeven -4.1%</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>ocQkotYQjj1jzVqq3ZyZtL4oRXcLK6zMuwLXqWRpump</t>
+          <t>GHnGviuMzqMoBx8NuZNN3X5QDkYA7mZBu3xVGoPNmVzT</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:39:52</t>
+          <t>2026-10-16 04:50:24</t>
         </is>
       </c>
       <c r="N2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:39:54</t>
+          <t>2026-10-16 04:50:25</t>
         </is>
       </c>
     </row>
@@ -915,61 +915,61 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Grokazon</t>
+          <t>Flying Tesla Roadster 2.0</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>GZON</t>
+          <t>FTR</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>LOST</t>
+          <t>WON</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>-0.9%</t>
+          <t>+24.4%</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>+7.4%</t>
+          <t>+68.5%</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>-0.9%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="H3" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.991037663</v>
+        <v>1.244047792</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>-0.008962337000000042</v>
+        <v>0.2440477919999999</v>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>watchdog breakeven -0.9%</t>
+          <t>trade-event ratchet-floor 24.4% (locked +25%, peak +68%)</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>8LwcuvF6drQ21pmhZm1qGZBdeLkLGHx2q9XHDV65pump</t>
+          <t>J5s6eTHv3ZhzG5X4LrEwbr1LgRoj5tSmsZDrxntMpump</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:39:54</t>
+          <t>2026-10-16 04:50:29</t>
         </is>
       </c>
       <c r="N3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:39:56</t>
+          <t>2026-10-16 04:50:31</t>
         </is>
       </c>
     </row>
@@ -979,63 +979,43 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>rivaly.fun</t>
+          <t>numen.cash</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>RIVALY</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>-7.0%</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>-7.0%</t>
-        </is>
-      </c>
+          <t>NUMEN</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="9" t="inlineStr"/>
       <c r="H4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="12" t="n">
-        <v>0.930309045</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>-0.069690955</v>
-      </c>
+      <c r="I4" s="10" t="inlineStr"/>
+      <c r="J4" s="10" t="inlineStr"/>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>watchdog stop-loss -7.0%</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="L4" s="10" t="inlineStr">
         <is>
-          <t>6N22dmEVa9Ky8ezvhm5FvCtTpFgd9fLBuSW9wSmwpump</t>
+          <t>GvEjB2Z24Hbq3Tf3F5e5vPgBpmV5p7YnL4SLDpoapump</t>
         </is>
       </c>
       <c r="M4" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:39:55</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:39:56</t>
-        </is>
-      </c>
+          <t>2026-10-16 04:50:31</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -1043,12 +1023,12 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Toly $1 Coin</t>
+          <t>p-null.si</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>p(null)</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
@@ -1071,12 +1051,12 @@
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>2dwa82kTNo8MXvj3K8wZqsx79h97pTXC2nCAfTkYpump</t>
+          <t>DuQU1Fi4KmT4cQgn1k1QYkqtYVEMRhEXbdijsipypump</t>
         </is>
       </c>
       <c r="M5" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:40:10</t>
+          <t>2026-10-16 04:50:37</t>
         </is>
       </c>
       <c r="N5" s="10" t="inlineStr"/>
@@ -1087,12 +1067,12 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Flying tesla skyster</t>
+          <t>Cuck Coding</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>FTS</t>
+          <t>Cuck</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -1115,386 +1095,18 @@
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t>3njQBDXmF4Z97u5BJzAzBRuMTMA89N3942i65pdLpump</t>
+          <t>4RrzBXWpbXbSsTNHxDxEjffrSzuG4HPoSLwPr7yVpump</t>
         </is>
       </c>
       <c r="M6" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:40:13</t>
+          <t>2026-10-16 04:50:41</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Baton Man</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>BatonMan</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>+30.1%</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>+48.5%</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <v>1.300951674</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>0.300951674</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>watchdog trailing-stop 30.1% (-12.4% from peak, tol=10%)</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>8f6htt8WT2qGau2T7MBXMW9NJXpcfFhTetdrcS2Rpump</t>
-        </is>
-      </c>
-      <c r="M7" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:17</t>
-        </is>
-      </c>
-      <c r="N7" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:18</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Ava Larps</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Ava</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L8" s="10" t="inlineStr">
-        <is>
-          <t>95yf3XvjpTzJfWAcqqvXhH5s4DS55tY1tiJ1iR9qpump</t>
-        </is>
-      </c>
-      <c r="M8" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:24</t>
-        </is>
-      </c>
-      <c r="N8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>ТamPad</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>ТamPad</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="10" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L9" s="10" t="inlineStr">
-        <is>
-          <t>DiGYfgNSzYsvN4zbjZa6NyjyNE95X2qkV32ML5thpump</t>
-        </is>
-      </c>
-      <c r="M9" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:51</t>
-        </is>
-      </c>
-      <c r="N9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>ТamPad</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>ТamPad</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>-1.8%</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>-0.8%</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="12" t="n">
-        <v>0.981940087</v>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>-0.01805991299999998</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>watchdog dead-coin -0.8% after 30s</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>FppJ8swha44WggXN2UG9mTKG1b35ACBUYhvMsdKWpump</t>
-        </is>
-      </c>
-      <c r="M10" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:56</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:41:26</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>amor</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>amor</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>+25.4%</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>+69.8%</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="12" t="n">
-        <v>1.253915268</v>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>0.2539152680000001</v>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>watchdog trailing-stop 25.4% (-26.2% from peak, tol=18%)</t>
-        </is>
-      </c>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>HuDj7pNgAcVXb7cEtPXJEQTqVQGQGkuHBTh7Djsopump</t>
-        </is>
-      </c>
-      <c r="M11" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:41:19</t>
-        </is>
-      </c>
-      <c r="N11" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:41:29</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>TESCREAL</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>TESCREAL</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="10" t="inlineStr"/>
-      <c r="K12" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L12" s="10" t="inlineStr">
-        <is>
-          <t>NZZY9SnqrMLHiHxoqnstLCsF7Lmr1rGF1Ba3HAEpump</t>
-        </is>
-      </c>
-      <c r="M12" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:41:25</t>
-        </is>
-      </c>
-      <c r="N12" s="10" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>DRAINLOVE</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>DRAINLOVE</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
-      <c r="G13" s="9" t="inlineStr"/>
-      <c r="H13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="10" t="inlineStr"/>
-      <c r="J13" s="10" t="inlineStr"/>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L13" s="10" t="inlineStr">
-        <is>
-          <t>9HmC4jXxkaFchQHQEy873oA3bCcpGziz1hW7aP14pump</t>
-        </is>
-      </c>
-      <c r="M13" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:41:34</t>
-        </is>
-      </c>
-      <c r="N13" s="10" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N13"/>
+  <autoFilter ref="A1:N6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1505,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1563,144 +1175,36 @@
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>2026-10-16 04:39:57</t>
+          <t>2026-10-16 04:50:34</t>
         </is>
       </c>
       <c r="B2" s="16" t="inlineStr">
         <is>
-          <t>SUPER INU</t>
+          <t>Flying Tesla Roadster 2.0</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>SINU</t>
+          <t>FTR2,0</t>
         </is>
       </c>
       <c r="D2" s="17" t="n">
-        <v>3.319804998249779</v>
+        <v>80.87747102079877</v>
       </c>
       <c r="E2" s="18" t="n">
-        <v>7919.615246532211</v>
+        <v>521.0370369380399</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
-          <t>1- Liquidity (LP tokens) Locked 3.32% | 2- Total Locked Liquidity $7.9K | BLOCK insider-whale 763,701,068 tokens (&gt;= 100,000,000); concentrated-holder 76.4% &gt;= 30%</t>
+          <t>1- Liquidity (LP tokens) Locked 80.88% | 2- Total Locked Liquidity $521 | BLOCK insider-whale 151,660,777 tokens (&gt;= 100,000,000)</t>
         </is>
       </c>
       <c r="G2" s="18" t="n">
-        <v>763701067.612466</v>
+        <v>151660777.334045</v>
       </c>
       <c r="H2" s="16" t="inlineStr">
         <is>
-          <t>3szhHxoagYbDNEEj35cmBxKr3iadFLrrSVyjjuwapump</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:12</t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>Phase Punk</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>PHASEPUNK</t>
-        </is>
-      </c>
-      <c r="D3" s="17" t="n">
-        <v>135.291892573446</v>
-      </c>
-      <c r="E3" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
-        <is>
-          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=15 &gt; 5</t>
-        </is>
-      </c>
-      <c r="G3" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="16" t="inlineStr">
-        <is>
-          <t>9KGZuyJ8UXokgREBFxGguA1hVVdUmBYwtTSaQbPMpump</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:19</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Up Side Down Tesla</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D4" s="17" t="n">
-        <v>135.291892573446</v>
-      </c>
-      <c r="E4" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK clone-ticker USDT; serial-deployer launches=38 &gt; 5</t>
-        </is>
-      </c>
-      <c r="G4" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="16" t="inlineStr">
-        <is>
-          <t>7vG48c29W1oAtAeUUpphLgQ2bDUWTiXokhrYF2zsX34p</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:40:41</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>niggi</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>niggi</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="n">
-        <v>135.291892573446</v>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=6 &gt; 5</t>
-        </is>
-      </c>
-      <c r="G5" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="16" t="inlineStr">
-        <is>
-          <t>3o1kTH57F6kuuhjcpMSuggQHRjxmThEri3iGnPXfpump</t>
+          <t>7WZMwGsTkRkGyHHcAyCA1bcS65eaAQrFMakUc1LVz6pE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add automatic connectivity monitoring for unattended runs
Norton killed the test program twice with no error of any kind, so the overnight run
now proves its own network health instead of relying on someone being awake to click
Allow in a popup.

- check_connectivity.py gains a --log mode: one silent probe, one timestamped line in
  reports/logs/connectivity.log, exit code 0/1.
- sweep_program.ps1 probes once whenever it starts a fresh instance, so a blocked
  firewall is recorded in program.log rather than showing up as a silent night of no
  trades.
- conn_watch.cmd + the SolanaBotConnWatch task probe every 15 minutes.

Verified: both RPC and the WebSocket trade stream reachable, and the twice-run monitor
logged two OK lines.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +37,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="009C5700"/>
     </font>
     <font>
       <b val="1"/>
@@ -45,12 +45,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C5700"/>
+      <color rgb="001F4E79"/>
+      <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="16"/>
+      <color rgb="009C0006"/>
     </font>
   </fonts>
   <fills count="6">
@@ -67,7 +67,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -77,7 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,14 +107,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -134,13 +134,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -619,7 +616,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -629,7 +626,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -639,7 +636,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -659,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -670,7 +667,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -682,7 +679,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+72.7%</t>
+          <t>+68.5%</t>
         </is>
       </c>
     </row>
@@ -694,7 +691,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>-2.1%</t>
+          <t>+0.0%</t>
         </is>
       </c>
     </row>
@@ -705,7 +702,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -715,7 +712,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>2.202809591</v>
+        <v>1.025194494</v>
       </c>
     </row>
     <row r="21">
@@ -725,7 +722,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>0.2028095909999998</v>
+        <v>0.02519449399999996</v>
       </c>
     </row>
     <row r="22">
@@ -754,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -851,63 +848,43 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Okay</t>
+          <t>Roadster Wif Wings</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>OKAY</t>
+          <t>RWW</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>LOST</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>-4.1%</t>
-        </is>
-      </c>
-      <c r="F2" s="9" t="inlineStr">
-        <is>
-          <t>+76.9%</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr">
-        <is>
-          <t>-4.1%</t>
-        </is>
-      </c>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="9" t="inlineStr"/>
       <c r="H2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="12" t="n">
-        <v>0.958761799</v>
-      </c>
-      <c r="J2" s="12" t="n">
-        <v>-0.04123820099999997</v>
-      </c>
+      <c r="I2" s="10" t="inlineStr"/>
+      <c r="J2" s="10" t="inlineStr"/>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>trade-event breakeven -4.1%</t>
+          <t>holding</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>GHnGviuMzqMoBx8NuZNN3X5QDkYA7mZBu3xVGoPNmVzT</t>
+          <t>6oJLFN6wVz562HyB3LJHHxa2cG3fPr1DhBpD1gJ9pump</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:50:24</t>
-        </is>
-      </c>
-      <c r="N2" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:50:25</t>
-        </is>
-      </c>
+          <t>2026-10-16 04:57:40</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -915,12 +892,12 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Flying Tesla Roadster 2.0</t>
+          <t>Crashed Tesla Roadster</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>FTR</t>
+          <t>CTR</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
@@ -930,7 +907,7 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>+24.4%</t>
+          <t>+2.5%</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
@@ -947,166 +924,34 @@
         <v>1</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>1.244047792</v>
+        <v>1.025194494</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>0.2440477919999999</v>
+        <v>0.02519449399999996</v>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>trade-event ratchet-floor 24.4% (locked +25%, peak +68%)</t>
+          <t>trade-event ratchet-floor 2.5% (locked +25%, peak +69%)</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>J5s6eTHv3ZhzG5X4LrEwbr1LgRoj5tSmsZDrxntMpump</t>
+          <t>5VtDTJVXmbGZFuWtY8R1hmQ7nHpTLXuYDrqGzLXdbtf1</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:50:29</t>
+          <t>2026-10-16 04:57:54</t>
         </is>
       </c>
       <c r="N3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:50:31</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>numen.cash</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>NUMEN</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
-      <c r="G4" s="9" t="inlineStr"/>
-      <c r="H4" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="10" t="inlineStr"/>
-      <c r="J4" s="10" t="inlineStr"/>
-      <c r="K4" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>GvEjB2Z24Hbq3Tf3F5e5vPgBpmV5p7YnL4SLDpoapump</t>
-        </is>
-      </c>
-      <c r="M4" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:50:31</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>p-null.si</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>p(null)</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
-      <c r="G5" s="9" t="inlineStr"/>
-      <c r="H5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="10" t="inlineStr"/>
-      <c r="J5" s="10" t="inlineStr"/>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>DuQU1Fi4KmT4cQgn1k1QYkqtYVEMRhEXbdijsipypump</t>
-        </is>
-      </c>
-      <c r="M5" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:50:37</t>
-        </is>
-      </c>
-      <c r="N5" s="10" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Cuck Coding</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Cuck</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="10" t="inlineStr"/>
-      <c r="J6" s="10" t="inlineStr"/>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>holding</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>4RrzBXWpbXbSsTNHxDxEjffrSzuG4HPoSLwPr7yVpump</t>
-        </is>
-      </c>
-      <c r="M6" s="10" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:50:41</t>
-        </is>
-      </c>
-      <c r="N6" s="10" t="inlineStr"/>
+          <t>2026-10-16 04:57:56</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:N3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1117,7 +962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1131,80 +976,116 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Coin</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>LP tokens locked %</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Total liquidity USD</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>Reasons</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Top holder tokens</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>Mint</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>2026-10-16 04:50:34</t>
-        </is>
-      </c>
-      <c r="B2" s="16" t="inlineStr">
-        <is>
-          <t>Flying Tesla Roadster 2.0</t>
-        </is>
-      </c>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>FTR2,0</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="n">
-        <v>80.87747102079877</v>
-      </c>
-      <c r="E2" s="18" t="n">
-        <v>521.0370369380399</v>
-      </c>
-      <c r="F2" s="16" t="inlineStr">
-        <is>
-          <t>1- Liquidity (LP tokens) Locked 80.88% | 2- Total Locked Liquidity $521 | BLOCK insider-whale 151,660,777 tokens (&gt;= 100,000,000)</t>
-        </is>
-      </c>
-      <c r="G2" s="18" t="n">
-        <v>151660777.334045</v>
-      </c>
-      <c r="H2" s="16" t="inlineStr">
-        <is>
-          <t>7WZMwGsTkRkGyHHcAyCA1bcS65eaAQrFMakUc1LVz6pE</t>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:57:46</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Crashing Tesla Roadster</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>CTR</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="n">
+        <v>135.291892573446</v>
+      </c>
+      <c r="E2" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=41 &gt; 5</t>
+        </is>
+      </c>
+      <c r="G2" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>GNS1QtQ6Af34GXV7jpbaRw8qocRzQAqiVaDvTrdeGXsr</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-16 04:57:48</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Tusla</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>TUSLA</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>135.291892573446</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=10 &gt; 5</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>GnHdHDdW6xaxRikhqUF6xPMfZAkwzABDHy1qcMdypump</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a read-only sweep status reporter and start the 2/5/8 stream
tools/sweep_status.ps1 prints, at any moment, which plan stage is done, which arm is
running and how far into its block it is, and how many blocks have been recorded. It
only reads, so it is safe to run while the sweep is working.

Also clears stale per-stage .out files left by earlier aborted attempts so the report
reflects the current run.
</commit_message>
<xml_diff>
--- a/reports/pumpfun_trades.xlsx
+++ b/reports/pumpfun_trades.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$N$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,7 +37,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C5700"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
@@ -48,12 +48,8 @@
       <color rgb="001F4E79"/>
       <sz val="16"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,17 +63,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -114,8 +105,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -135,9 +126,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -616,7 +607,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -626,7 +617,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -636,7 +627,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -656,7 +647,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -667,7 +658,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -679,7 +670,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+68.5%</t>
+          <t>+4.1%</t>
         </is>
       </c>
     </row>
@@ -691,7 +682,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-1.9%</t>
         </is>
       </c>
     </row>
@@ -702,7 +693,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -712,7 +703,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1.025194494</v>
+        <v>5.70328915</v>
       </c>
     </row>
     <row r="21">
@@ -722,7 +713,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>0.02519449399999996</v>
+        <v>-0.2967108500000002</v>
       </c>
     </row>
     <row r="22">
@@ -751,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -848,43 +839,63 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Roadster Wif Wings</t>
+          <t>Roadster League</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>RWW</t>
+          <t>RDSTR</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
-      <c r="G2" s="9" t="inlineStr"/>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>-5.9%</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
       <c r="H2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="10" t="inlineStr"/>
-      <c r="J2" s="10" t="inlineStr"/>
+      <c r="I2" s="12" t="n">
+        <v>0.94128804</v>
+      </c>
+      <c r="J2" s="12" t="n">
+        <v>-0.05871196000000001</v>
+      </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>holding</t>
+          <t>watchdog stop-loss -4.0%</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>6oJLFN6wVz562HyB3LJHHxa2cG3fPr1DhBpD1gJ9pump</t>
+          <t>9VEBn4L7TWDKh1hFpuQfTJZfr4bZpooGnDnXQP7Jpump</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:57:40</t>
-        </is>
-      </c>
-      <c r="N2" s="10" t="inlineStr"/>
+          <t>2026-10-16 05:22:55</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:22:56</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -892,27 +903,27 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Crashed Tesla Roadster</t>
+          <t>ba-bump</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>CTR</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>WON</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>+2.5%</t>
+          <t>BABUMP</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>-5.9%</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>+68.5%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -924,34 +935,290 @@
         <v>1</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>1.025194494</v>
+        <v>0.94128804</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>0.02519449399999996</v>
+        <v>-0.05871196000000001</v>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>trade-event ratchet-floor 2.5% (locked +25%, peak +69%)</t>
+          <t>watchdog stop-loss -4.0%</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>5VtDTJVXmbGZFuWtY8R1hmQ7nHpTLXuYDrqGzLXdbtf1</t>
+          <t>Fdxu4ssBWHeq6wjioCHKZSdZEiVh2pmLLBa9aEprpump</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:57:54</t>
+          <t>2026-10-16 05:22:57</t>
         </is>
       </c>
       <c r="N3" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16 04:57:56</t>
+          <t>2026-10-16 05:22:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Roadster League</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>RL</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>WON</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>+7.1%</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>+24.7%</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>1.071451193</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>0.07145119299999991</v>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>trade-event trailing-stop 9.3% (-12.4% from peak, tol=10%)</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>DptdbbFwkLbKRCriN2sujYZkun7ZR7LfmSuocXgapump</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:22:58</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Roadster League</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>RL</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>-5.9%</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>0.94128804</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-0.05871196000000001</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>watchdog stop-loss -4.0%</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>6mtbYUmDMezp5KytZhZ6r25SQjckxupHkoWK7qnQpump</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:00</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Roadster League</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>RL</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>-5.9%</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>0.94128804</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>-0.05871196000000001</v>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>watchdog stop-loss -4.0%</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>6zFh6gadfmR2iUhVGXZhJ3wgwEUanZ4i4VS9ZBFjpump</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:14</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Halo.fun</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>HALO</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>-13.3%</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>-11.6%</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>0.866685797</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>-0.133314203</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>watchdog stop-loss -11.6%</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>6vAYQrLWb4kKRGkDGEV6cVXWRvF273WA3XhXcv4Qpump</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:15</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:16</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N3"/>
+  <autoFilter ref="A1:N7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -962,7 +1229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1020,17 +1287,17 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>2026-10-16 04:57:46</t>
+          <t>2026-10-16 05:23:06</t>
         </is>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Crashing Tesla Roadster</t>
+          <t>Roadster League</t>
         </is>
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>CTR</t>
+          <t>RL</t>
         </is>
       </c>
       <c r="D2" s="16" t="n">
@@ -1041,7 +1308,7 @@
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=41 &gt; 5</t>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=6 &gt; 5</t>
         </is>
       </c>
       <c r="G2" s="17" t="n">
@@ -1049,24 +1316,24 @@
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>GNS1QtQ6Af34GXV7jpbaRw8qocRzQAqiVaDvTrdeGXsr</t>
+          <t>BmVRs1bTmsNQxCPY7ZafqGFsmsT1f8crJS2Xa2U3pump</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>2026-10-16 04:57:48</t>
+          <t>2026-10-16 05:23:12</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Tusla</t>
+          <t>Roadster League</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>TUSLA</t>
+          <t>RL</t>
         </is>
       </c>
       <c r="D3" s="16" t="n">
@@ -1077,15 +1344,87 @@
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK serial-deployer launches=10 &gt; 5</t>
+          <t>1- Liquidity (LP tokens) Locked 135.29% | 2- Total Locked Liquidity $0 | BLOCK insider-whale 153,285,714 tokens (&gt;= 100,000,000); sniper-bundle 10 wallets besides LP</t>
         </is>
       </c>
       <c r="G3" s="17" t="n">
-        <v>0</v>
+        <v>153285714.285714</v>
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>GnHdHDdW6xaxRikhqUF6xPMfZAkwzABDHy1qcMdypump</t>
+          <t>Dv8Z4Mnmq6wsPF3Y82MTDGSXMZVnQh9rL5rq9u2Dpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:17</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Roadster League</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>RL</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>77.32066653540991</v>
+      </c>
+      <c r="E4" s="17" t="n">
+        <v>636.98458242588</v>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 77.32% | 2- Total Locked Liquidity $637 | BLOCK sniper-bundle 9 wallets besides LP</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="n">
+        <v>35804181.905251</v>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>arsE5wWTdHtFso8Pd5BM8wQ5xCmpKrA16Zm4YY2pump</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-16 05:23:19</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Roadster League</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>RL</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>71.51749630032745</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>843.44000010543</v>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>1- Liquidity (LP tokens) Locked 71.52% | 2- Total Locked Liquidity $843 | BLOCK sniper-bundle 14 wallets besides LP</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>59172794.117647</v>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>HvcX5VL5SpWX6yQvJor65Jzf2xKcTgvr11Nq3HUNpump</t>
         </is>
       </c>
     </row>

</xml_diff>